<commit_message>
daily log update: 2026-08-13
</commit_message>
<xml_diff>
--- a/12619762_Jasika_Pathania_Activity_Filled.xlsx
+++ b/12619762_Jasika_Pathania_Activity_Filled.xlsx
@@ -466,7 +466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A39"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
   </cols>
@@ -721,7 +721,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N415"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="6"/>

</xml_diff>

<commit_message>
daily log update: 2026-08-14
</commit_message>
<xml_diff>
--- a/12619762_Jasika_Pathania_Activity_Filled.xlsx
+++ b/12619762_Jasika_Pathania_Activity_Filled.xlsx
@@ -466,7 +466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A39"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
   </cols>
@@ -721,7 +721,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N415"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="6"/>

</xml_diff>